<commit_message>
design: C6 1 nF -> 10 nF (drawing RGX-2-100 Rev E, spec RGX-2-001 Rev D)
The shell-speed wire runs beside PWM-switched phase leads, and wheel
speed now feeds the slip regulator directly. R6*C6 = 10 us filters
us-scale spikes in hardware (a 1 us, 5 V spike reaches GP13 at ~0.5 V);
the rising edge through R5+R6 is 110 us, ~1 % of a half-period at
60 km/h, and the period measurement is unaffected.

- Drawing Rev E: C6 parts-list entry, title blocks, revision history.
- Spec Rev D: C6 row in the component schedule; header.
- BOM: C6 in the capacitor line, header references; the queued Higo W1
  change moves from Rev E to Rev F.
- READMEs, RGX-2-003 header, hardware-design note, decision log entry,
  design package zip.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LUoDci9bVDi6EYCYAJA33y
</commit_message>
<xml_diff>
--- a/design/RGX-2-002-BOM.xlsx
+++ b/design/RGX-2-002-BOM.xlsx
@@ -42,7 +42,7 @@
     <t>ReGenX v2 — Bill of Materials   ·   RGX-2-002 Rev A</t>
   </si>
   <si>
-    <t>Against RGX-2-001 Rev C / RGX-2-100 Rev D  ·  2026-08-02.  Prices approximate CAD, August 2026, before tax/shipping — blue cells are editable estimates; update them after quoting. Sourcing assumes delivery to Ontario.</t>
+    <t>Against RGX-2-001 Rev D / RGX-2-100 Rev E  ·  2026-09-29.  Prices approximate CAD, August 2026, before tax/shipping — blue cells are editable estimates; update them after quoting. Sourcing assumes delivery to Ontario.</t>
   </si>
   <si>
     <t>Summary (CAD)</t>
@@ -447,7 +447,7 @@
     <t>Ceramic caps</t>
   </si>
   <si>
-    <t>2x 100 nF &gt;=16 V X7R; 1 nF &gt;=50 V C0G</t>
+    <t>2x 100 nF &gt;=16 V X7R; 10 nF &gt;=50 V C0G</t>
   </si>
   <si>
     <t>Ceramic assortment kit - Amazon.ca</t>
@@ -552,10 +552,10 @@
     <t>Single 9-pin Higo Z910, NOT the separate 6-way J1 drawn on Sheet 3</t>
   </si>
   <si>
-    <t>W1 redefined as Z910 splitter - electrically identical. Queued as drawing Rev E. Pinouts vary: continuity-map before power</t>
-  </si>
-  <si>
-    <t>Drawing Rev E</t>
+    <t>W1 redefined as Z910 splitter - electrically identical. Queued as drawing Rev F. Pinouts vary: continuity-map before power</t>
+  </si>
+  <si>
+    <t>Drawing Rev F</t>
   </si>
   <si>
     <t>Back-EMF, coasting</t>

</xml_diff>

<commit_message>
design: drawing RGX-2-100 Rev F, spec RGX-2-001 Rev E
- U2's ground return lands on the GND pin of A1's UART connector, the
  reference of the UART signals, instead of the V- star. A1's V- pigtail
  carries the battery current, and its drop no longer sits between the
  two grounds. Still the only U2 ground path. +5V_RTN drawn on sheet 3.
- Sheet 3 NOTE 9: UART_TX, UART_RX, +5V and +5V_RTN run as one twisted
  bundle. The star notes on sheets 1 and 2 now name power grounds.
- Sheet 3 NOTE 7 and spec section 10 item 6 (VSYS logging) withdrawn.
- J1 redrawn as M1's single Higo Z910 cable, pins by continuity map;
  W1 is the Z910 splitter (queued since RGX-2-002 Rev A).
- BOM header and queued-change rows updated; design package rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LUoDci9bVDi6EYCYAJA33y
</commit_message>
<xml_diff>
--- a/design/RGX-2-002-BOM.xlsx
+++ b/design/RGX-2-002-BOM.xlsx
@@ -42,7 +42,7 @@
     <t>ReGenX v2 — Bill of Materials   ·   RGX-2-002 Rev A</t>
   </si>
   <si>
-    <t>Against RGX-2-001 Rev D / RGX-2-100 Rev E  ·  2026-09-29.  Prices approximate CAD, August 2026, before tax/shipping — blue cells are editable estimates; update them after quoting. Sourcing assumes delivery to Ontario.</t>
+    <t>Against RGX-2-001 Rev E / RGX-2-100 Rev F  ·  2026-09-29.  Prices approximate CAD, August 2026, before tax/shipping — blue cells are editable estimates; update them after quoting. Sourcing assumes delivery to Ontario.</t>
   </si>
   <si>
     <t>Summary (CAD)</t>
@@ -549,13 +549,13 @@
     <t>Cable / W1</t>
   </si>
   <si>
-    <t>Single 9-pin Higo Z910, NOT the separate 6-way J1 drawn on Sheet 3</t>
-  </si>
-  <si>
-    <t>W1 redefined as Z910 splitter - electrically identical. Queued as drawing Rev F. Pinouts vary: continuity-map before power</t>
-  </si>
-  <si>
-    <t>Drawing Rev F</t>
+    <t>Single 9-pin Higo Z910, drawn as J1 from drawing Rev F</t>
+  </si>
+  <si>
+    <t>W1 is the Z910 splitter - electrically identical. Drawn at Rev F. Pinouts vary: continuity-map before power</t>
+  </si>
+  <si>
+    <t>Done at drawing Rev F</t>
   </si>
   <si>
     <t>Back-EMF, coasting</t>

</xml_diff>

<commit_message>
G020 constants from published data; back-EMF crossover corrected
- MOTOR_FLUX_WB 0.020 -> 0.0162 Wb: from Bafang's no-load 245 rpm at
  36 V for the 26-28 in winding (10 pole pairs, 5:1), with line-to-line
  back-EMF equal to the supply at no load.
- MOTOR_R_OHM 0.30 -> 0.25 ohm per phase: ~0.5 ohm phase-to-phase
  reported for the SWX02. The speed droop to the rated 205 rpm at 80 %
  efficiency gives ~0.34 ohm, an upper bound.
- The yield cap barely moves: 5.3 A at 3 km/h, 18 A at 10 km/h, 35 A
  at 20 km/h.
- kV from the no-load speed is ~6.8 wheel-rpm/V, not 5.56 (which used the
  loaded speed), so the back-EMF crossover is 10.9 / 34 / 39 km/h at
  12.7 / 40 / 45.4 V, not 8.9 / 28 / 31.8. BOM compatibility sheet
  updated (RGX-2-002 Rev B), components note and decision log too.

Both constants stay [BENCH]: the VESC's FOC motor detection replaces them.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LUoDci9bVDi6EYCYAJA33y
</commit_message>
<xml_diff>
--- a/design/RGX-2-002-BOM.xlsx
+++ b/design/RGX-2-002-BOM.xlsx
@@ -39,7 +39,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="286">
   <si>
-    <t>ReGenX v2 — Bill of Materials   ·   RGX-2-002 Rev A</t>
+    <t>ReGenX v2 — Bill of Materials   ·   RGX-2-002 Rev B</t>
   </si>
   <si>
     <t>Against RGX-2-001 Rev E / RGX-2-100 Rev F  ·  2026-09-29.  Prices approximate CAD, August 2026, before tax/shipping — blue cells are editable estimates; update them after quoting. Sourcing assumes delivery to Ontario.</t>
@@ -492,7 +492,7 @@
     <t>Compatibility verification — computed against RGX-2-001 Rev C</t>
   </si>
   <si>
-    <t>G020 research-confirmed: 20 magnets (10 pole pairs), 5:1 single-stage, 6-magnet shell speed sensor, ~200 rpm @ 36 V =&gt; kV_wheel ~5.56 rpm/V. Measured kV (spec s11 gate 2) replaces the estimate.</t>
+    <t>G020 research-confirmed: 20 magnets (10 pole pairs), 5:1 single-stage, 6-magnet shell speed sensor, no-load 245 rpm @ 36 V (26-28 in winding) =&gt; kV_wheel ~6.8 rpm/V. Measured kV (spec s11 gate 2) replaces the estimate.</t>
   </si>
   <si>
     <t>Area</t>
@@ -570,7 +570,7 @@
     <t>Back-EMF vs bank 12.7 V (rest)</t>
   </si>
   <si>
-    <t>Crossover 8.9 km/h wheel speed during braking</t>
+    <t>Crossover 10.9 km/h wheel speed during braking</t>
   </si>
   <si>
     <t>This is regen working as intended</t>
@@ -579,19 +579,19 @@
     <t>Back-EMF vs bank 40 V (full)</t>
   </si>
   <si>
-    <t>Crossover 28.0 km/h</t>
-  </si>
-  <si>
-    <t>Braking below 28 km/h can NEVER overcharge a full bank, even via body diodes with A1 faulted</t>
+    <t>Crossover 34.3 km/h</t>
+  </si>
+  <si>
+    <t>Braking below 34 km/h can NEVER overcharge a full bank, even via body diodes with A1 faulted</t>
   </si>
   <si>
     <t>Back-EMF vs bank 45.4 V (abs)</t>
   </si>
   <si>
-    <t>Crossover 31.8 km/h</t>
-  </si>
-  <si>
-    <t>Exposure: braking &gt;32 km/h + full bank + faulted A1. Control law must taper full-bank regen to zero above ~28 km/h. Carrier slip reduces rotor speed and therefore back-EMF, softening the exposure further</t>
+    <t>Crossover 38.9 km/h</t>
+  </si>
+  <si>
+    <t>Exposure: braking &gt;39 km/h + full bank + faulted A1. Control law must taper full-bank regen to zero above ~34 km/h. Carrier slip reduces rotor speed and therefore back-EMF, softening the exposure further</t>
   </si>
   <si>
     <t>Control-law req</t>
@@ -762,7 +762,7 @@
     <t>M1 kV</t>
   </si>
   <si>
-    <t>Drill-spin, open-circuit phase voltage vs rpm - replaces 5.56 rpm/V estimate and re-derives crossover table</t>
+    <t>Drill-spin, open-circuit phase voltage vs rpm - replaces 6.8 rpm/V estimate and re-derives crossover table</t>
   </si>
   <si>
     <t>Spec s11 gate 2</t>
@@ -816,7 +816,7 @@
     <t>Control law (deferred phase)</t>
   </si>
   <si>
-    <t>Full-bank regen tapered to zero above ~28 km/h; wheel rpm = ERPM / 50</t>
+    <t>Full-bank regen tapered to zero above ~34 km/h; wheel rpm = ERPM / 50</t>
   </si>
   <si>
     <t>Sources — research behind selections and compatibility findings</t>

</xml_diff>